<commit_message>
Add stats and processing
</commit_message>
<xml_diff>
--- a/processed_data/barcelona.xlsx
+++ b/processed_data/barcelona.xlsx
@@ -593,7 +593,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>[['Raphinha', "7'"], ['Ferran Torres', "23'"], ['Lamine Yamal', "90+4'"]]</t>
+          <t>[[Raphinha,7],[Ferran Torres,23],[Lamine Yamal,90+4]]</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -692,7 +692,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>[['Pedri', "49'"], ['Ferran Torres', "52'"], ['Unai Elgezabal', "90+1' (GEC)"]]</t>
+          <t>[[Pedri,49],[Ferran Torres,52],[Unai Elgezabal,90+1 (GEC)]]</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -727,7 +727,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>[['Iván Romero', "15'"], ['José Luis Morales Nogales', "45+7' (P)"]]</t>
+          <t>[[Iván Romero,15],[José Luis Morales Nogales,45+7 (P)]]</t>
         </is>
       </c>
       <c r="T3" t="n">
@@ -791,7 +791,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>[['Lamine Yamal', "40' (P)"]]</t>
+          <t>[[Lamine Yamal,40 (P)]]</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -826,7 +826,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>[['Fran Pérez Martínez', "67'"]]</t>
+          <t>[[Fran Pérez Martínez,67]]</t>
         </is>
       </c>
       <c r="T4" t="n">
@@ -890,7 +890,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>[['Fermín López Marín', "29',", "56'"], ['Raphinha', "53',", "66'"], ['Robert Lewandowski', "76',", "86'"]]</t>
+          <t>[[Fermín López Marín,29,56],[Raphinha,53,66],[Robert Lewandowski,76,86]]</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -989,7 +989,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>[['Marcus Rashford', "58',", "67'"]]</t>
+          <t>[[Marcus Rashford,58,67]]</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>[['Anthony Gordon', "90'"]]</t>
+          <t>[[Anthony Gordon,90]]</t>
         </is>
       </c>
       <c r="T6" t="n">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>[['Ferran Torres', "15',", "34'"], ['Dani Olmo', "62'"]]</t>
+          <t>[[Ferran Torres,15,34],[Dani Olmo,62]]</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>[['Eric García', "56'"], ['Robert Lewandowski', "70'"], ['Ronald Araújo', "88'"]]</t>
+          <t>[[Eric García,56],[Robert Lewandowski,70],[Ronald Araújo,88]]</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>[['Alberto Reina', "33'"]]</t>
+          <t>[[Alberto Reina,33]]</t>
         </is>
       </c>
       <c r="T8" t="n">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>[['Jules Koundé', "43'"], ['Robert Lewandowski', "59'"]]</t>
+          <t>[[Jules Koundé,43],[Robert Lewandowski,59]]</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>[['Álvaro Odriozola', "31'"]]</t>
+          <t>[[Álvaro Odriozola,31]]</t>
         </is>
       </c>
       <c r="T9" t="n">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>[['Ferran Torres', "19'"]]</t>
+          <t>[[Ferran Torres,19]]</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>[['Senny Mayulu', "38'"], ['Gonçalo Ramos', "90'"]]</t>
+          <t>[[Senny Mayulu,38],[Gonçalo Ramos,90]]</t>
         </is>
       </c>
       <c r="T10" t="n">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>[['Marcus Rashford', "45+7'"]]</t>
+          <t>[[Marcus Rashford,45+7]]</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>[['Alexis Sánchez', "13' (P)"], ['Isaac Romero', "37'"], ['José Ángel Carmona', "90'"], ['Akor Adams', "90+6'"]]</t>
+          <t>[[Alexis Sánchez,13 (P)],[Isaac Romero,37],[José Ángel Carmona,90],[Akor Adams,90+6]]</t>
         </is>
       </c>
       <c r="T11" t="n">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>[['Pedri', "13'"], ['Ronald Araújo', "90+3'"]]</t>
+          <t>[[Pedri,13],[Ronald Araújo,90+3]]</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>[['Axel Witsel', "20'"]]</t>
+          <t>[[Axel Witsel,20]]</t>
         </is>
       </c>
       <c r="T12" t="n">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>[['Fermín López Marín', "7',", "39',", "76'"], ['Lamine Yamal', "68' (P)"], ['Marcus Rashford', "74',", "79'"]]</t>
+          <t>[[Fermín López Marín,7,39,76],[Lamine Yamal,68 (P)],[Marcus Rashford,74,79]]</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -1713,7 +1713,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>[['Ayoub El Kaabi', "53' (P)"]]</t>
+          <t>[[Ayoub El Kaabi,53 (P)]]</t>
         </is>
       </c>
       <c r="T13" t="n">
@@ -1777,7 +1777,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>[['Fermín López Marín', "38'"]]</t>
+          <t>[[Fermín López Marín,38]]</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>[['Kylian Mbappé', "22'"], ['Jude Bellingham', "43'"]]</t>
+          <t>[[Kylian Mbappé,22],[Jude Bellingham,43]]</t>
         </is>
       </c>
       <c r="T14" t="n">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>[['Lamine Yamal', "9'"], ['Ferran Torres', "12'"], ['Marcus Rashford', "61'"]]</t>
+          <t>[[Lamine Yamal,9],[Ferran Torres,12],[Marcus Rashford,61]]</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>[['Rafa Mir', "42'"]]</t>
+          <t>[[Rafa Mir,42]]</t>
         </is>
       </c>
       <c r="T15" t="n">
@@ -1971,7 +1971,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>[['Ferran Torres', "8'"], ['Lamine Yamal', "61'"], ['Christos Tzolis', "77' (GEC)"]]</t>
+          <t>[[Ferran Torres,8],[Lamine Yamal,61],[Christos Tzolis,77 (GEC)]]</t>
         </is>
       </c>
       <c r="I16" t="n">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>[['Nicolò Tresoldi', "6'"], ['Carlos Forbs', "17',", "63'"]]</t>
+          <t>[[Nicolò Tresoldi,6],[Carlos Forbs,17,63]]</t>
         </is>
       </c>
       <c r="T16" t="n">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>[['Robert Lewandowski', "10' (P),", "37',", "73'"], ['Lamine Yamal', "45+4'"]]</t>
+          <t>[[Robert Lewandowski,10 (P),37,73],[Lamine Yamal,45+4]]</t>
         </is>
       </c>
       <c r="I17" t="n">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>[['Sergio Carreira', "11'"], ['Borja Iglesias', "43'"]]</t>
+          <t>[[Sergio Carreira,11],[Borja Iglesias,43]]</t>
         </is>
       </c>
       <c r="T17" t="n">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>[['Robert Lewandowski', "4'"], ['Ferran Torres', "45+3',", "90'"], ['Fermín López Marín', "48'"]]</t>
+          <t>[[Robert Lewandowski,4],[Ferran Torres,45+3,90],[Fermín López Marín,48]]</t>
         </is>
       </c>
       <c r="I18" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>[['Jules Koundé', "27' (GEC)"], ['Estêvão Willian', "55'"], ['Liam Delap', "73'"]]</t>
+          <t>[[Jules Koundé,27 (GEC)],[Estêvão Willian,55],[Liam Delap,73]]</t>
         </is>
       </c>
       <c r="T19" t="n">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>[['Lamine Yamal', "8'"], ['Dani Olmo', "26',", "90+3'"]]</t>
+          <t>[[Lamine Yamal,8],[Dani Olmo,26,90+3]]</t>
         </is>
       </c>
       <c r="I20" t="n">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>[['Pablo Ibáñez Lumbreras', "1'"]]</t>
+          <t>[[Pablo Ibáñez Lumbreras,1]]</t>
         </is>
       </c>
       <c r="T20" t="n">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>[['Raphinha', "26'"], ['Dani Olmo', "65'"], ['Ferran Torres', "90+7'"]]</t>
+          <t>[[Raphinha,26],[Dani Olmo,65],[Ferran Torres,90+7]]</t>
         </is>
       </c>
       <c r="I21" t="n">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>[['Álex Baena', "19'"]]</t>
+          <t>[[Álex Baena,19]]</t>
         </is>
       </c>
       <c r="T21" t="n">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>[['Ferran Torres', "11',", "13',", "40'"], ['Roony Bardghji', "31'"], ['Lamine Yamal', "59' (P)"]]</t>
+          <t>[[Ferran Torres,11,13,40],[Roony Bardghji,31],[Lamine Yamal,59 (P)]]</t>
         </is>
       </c>
       <c r="I22" t="n">
@@ -2600,7 +2600,7 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>[['Antony dos Santos', "6'"], ['Diego Llorente', "85'"], ['Cucho Hernández', "90' (P)"]]</t>
+          <t>[[Antony dos Santos,6],[Diego Llorente,85],[Cucho Hernández,90 (P)]]</t>
         </is>
       </c>
       <c r="T22" t="n">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>[['Jules Koundé', "50',", "53'"]]</t>
+          <t>[[Jules Koundé,50,53]]</t>
         </is>
       </c>
       <c r="I23" t="n">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>[['Ansgar Knauff', "21'"]]</t>
+          <t>[[Ansgar Knauff,21]]</t>
         </is>
       </c>
       <c r="T23" t="n">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>[['Raphinha', "70',", "86'"]]</t>
+          <t>[[Raphinha,70,86]]</t>
         </is>
       </c>
       <c r="I24" t="n">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>[['Andreas Christensen', "76'"], ['Marcus Rashford', "90'"]]</t>
+          <t>[[Andreas Christensen,76],[Marcus Rashford,90]]</t>
         </is>
       </c>
       <c r="I25" t="n">
@@ -2957,7 +2957,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>[['Raphinha', "12' (P)"], ['Lamine Yamal', "63'"]]</t>
+          <t>[[Raphinha,12 (P)],[Lamine Yamal,63]]</t>
         </is>
       </c>
       <c r="I26" t="n">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>[['Dani Olmo', "86'"], ['Robert Lewandowski', "90'"]]</t>
+          <t>[[Dani Olmo,86],[Robert Lewandowski,90]]</t>
         </is>
       </c>
       <c r="I27" t="n">
@@ -3151,7 +3151,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>[['Ferran Torres', "22'"], ['Fermín López Marín', "30'"], ['Roony Bardghji', "34'"], ['Raphinha', "38',", "52'"]]</t>
+          <t>[[Ferran Torres,22],[Fermín López Marín,30],[Roony Bardghji,34],[Raphinha,38,52]]</t>
         </is>
       </c>
       <c r="I28" t="n">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>[['Raphinha', "36',", "73'"], ['Robert Lewandowski', "45+4'"]]</t>
+          <t>[[Raphinha,36,73],[Robert Lewandowski,45+4]]</t>
         </is>
       </c>
       <c r="I29" t="n">
@@ -3281,7 +3281,7 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>[['Vinícius Júnior', "45+2'"], ['Gonzalo García Torres', "45+6'"]]</t>
+          <t>[[Vinícius Júnior,45+2],[Gonzalo García Torres,45+6]]</t>
         </is>
       </c>
       <c r="T29" t="n">
@@ -3345,7 +3345,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>[['Ferran Torres', "66'"], ['Lamine Yamal', "90+6'"]]</t>
+          <t>[[Ferran Torres,66],[Lamine Yamal,90+6]]</t>
         </is>
       </c>
       <c r="I30" t="n">
@@ -3444,7 +3444,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>[['Marcus Rashford', "70'"]]</t>
+          <t>[[Marcus Rashford,70]]</t>
         </is>
       </c>
       <c r="I31" t="n">
@@ -3479,7 +3479,7 @@
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>[['Mikel Oyarzabal', "32'"], ['Gonçalo Guedes', "71'"]]</t>
+          <t>[[Mikel Oyarzabal,32],[Gonçalo Guedes,71]]</t>
         </is>
       </c>
       <c r="T31" t="n">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>[['Fermín López Marín', "34',", "42'"], ['Dani Olmo', "63'"], ['Robert Lewandowski', "70'"]]</t>
+          <t>[[Fermín López Marín,34,42],[Dani Olmo,63],[Robert Lewandowski,70]]</t>
         </is>
       </c>
       <c r="I32" t="n">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>[['Vasil Kušej', "10'"], ['Robert Lewandowski', "44' (GEC)"]]</t>
+          <t>[[Vasil Kušej,10],[Robert Lewandowski,44 (GEC)]]</t>
         </is>
       </c>
       <c r="T32" t="n">
@@ -3642,7 +3642,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>[['Dani Olmo', "52'"], ['Raphinha', "57'"], ['Lamine Yamal', "73'"]]</t>
+          <t>[[Dani Olmo,52],[Raphinha,57],[Lamine Yamal,73]]</t>
         </is>
       </c>
       <c r="I33" t="n">
@@ -3741,7 +3741,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>[['Robert Lewandowski', "48'"], ['Lamine Yamal', "60'"], ['Raphinha', "69' (P)"], ['Marcus Rashford', "85'"]]</t>
+          <t>[[Robert Lewandowski,48],[Lamine Yamal,60],[Raphinha,69 (P)],[Marcus Rashford,85]]</t>
         </is>
       </c>
       <c r="I34" t="n">
@@ -3776,7 +3776,7 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>[['Viktor Daðason', "4'"]]</t>
+          <t>[[Viktor Daðason,4]]</t>
         </is>
       </c>
       <c r="T34" t="n">
@@ -3840,7 +3840,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>[['Lamine Yamal', "6'"], ['Ferran Torres', "40'"], ['Marcus Rashford', "72'"]]</t>
+          <t>[[Lamine Yamal,6],[Ferran Torres,40],[Marcus Rashford,72]]</t>
         </is>
       </c>
       <c r="I35" t="n">
@@ -3875,7 +3875,7 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>[['Álvaro Rodríguez Muñoz', "29'"]]</t>
+          <t>[[Álvaro Rodríguez Muñoz,29]]</t>
         </is>
       </c>
       <c r="T35" t="n">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>[['Lamine Yamal', "39'"], ['Ronald Araújo', "56'"]]</t>
+          <t>[[Lamine Yamal,39],[Ronald Araújo,56]]</t>
         </is>
       </c>
       <c r="I36" t="n">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>[['Javier Moreno Arrones', "87'"]]</t>
+          <t>[[Javier Moreno Arrones,87]]</t>
         </is>
       </c>
       <c r="T36" t="n">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>[['Robert Lewandowski', "29'"], ['Lamine Yamal', "61'"], ['Marc Bernal', "83'"]]</t>
+          <t>[[Robert Lewandowski,29],[Lamine Yamal,61],[Marc Bernal,83]]</t>
         </is>
       </c>
       <c r="I37" t="n">
@@ -4172,7 +4172,7 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>[['Eric García', "7' (GEC)"], ['Antoine Griezmann', "14'"], ['Ademola Lookman', "33'"], ['Julián Alvarez', "45+2'"]]</t>
+          <t>[[Eric García,7 (GEC)],[Antoine Griezmann,14],[Ademola Lookman,33],[Julián Alvarez,45+2]]</t>
         </is>
       </c>
       <c r="T38" t="n">
@@ -4236,7 +4236,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>[['Pau Cubarsí', "59'"]]</t>
+          <t>[[Pau Cubarsí,59]]</t>
         </is>
       </c>
       <c r="I39" t="n">
@@ -4271,7 +4271,7 @@
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>[['Thomas Lemar', "62'"], ['Fran Beltrán', "86'"]]</t>
+          <t>[[Thomas Lemar,62],[Fran Beltrán,86]]</t>
         </is>
       </c>
       <c r="T39" t="n">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>[['Marc Bernal', "4'"], ['Frenkie de Jong', "32'"], ['Fermín López Marín', "81'"]]</t>
+          <t>[[Marc Bernal,4],[Frenkie de Jong,32],[Fermín López Marín,81]]</t>
         </is>
       </c>
       <c r="I40" t="n">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>[['Lamine Yamal', "28',", "37',", "69'"], ['Robert Lewandowski', "90+1'"]]</t>
+          <t>[[Lamine Yamal,28,37,69],[Robert Lewandowski,90+1]]</t>
         </is>
       </c>
       <c r="I41" t="n">
@@ -4469,7 +4469,7 @@
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>[['Pape Gueye', "49'"]]</t>
+          <t>[[Pape Gueye,49]]</t>
         </is>
       </c>
       <c r="T41" t="n">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>[['Marc Bernal', "29',", "72'"], ['Raphinha', "45+5' (P)"]]</t>
+          <t>[[Marc Bernal,29,72],[Raphinha,45+5 (P)]]</t>
         </is>
       </c>
       <c r="I42" t="n">
@@ -4632,7 +4632,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>[['Lamine Yamal', "68'"]]</t>
+          <t>[[Lamine Yamal,68]]</t>
         </is>
       </c>
       <c r="I43" t="n">
@@ -4731,7 +4731,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>[['Lamine Yamal', "90+6' (P)"]]</t>
+          <t>[[Lamine Yamal,90+6 (P)]]</t>
         </is>
       </c>
       <c r="I44" t="n">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>[['Harvey Barnes', "86'"]]</t>
+          <t>[[Harvey Barnes,86]]</t>
         </is>
       </c>
       <c r="T44" t="n">
@@ -4830,7 +4830,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>[['Raphinha', "9' (P),", "21' (P),", "51'"], ['Dani Olmo', "38'"], ['João Cancelo', "60'"]]</t>
+          <t>[[Raphinha,9 (P),21 (P),51],[Dani Olmo,38],[João Cancelo,60]]</t>
         </is>
       </c>
       <c r="I45" t="n">
@@ -4865,7 +4865,7 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>[['Oso', "45+4'"], ['Djibril Sow', "90+2'"]]</t>
+          <t>[[Oso,45+4],[Djibril Sow,90+2]]</t>
         </is>
       </c>
       <c r="T45" t="n">
@@ -4929,7 +4929,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>[['Raphinha', "6',", "72'"], ['Marc Bernal', "18'"], ['Lamine Yamal', "45+7' (P)"], ['Fermín López Marín', "51'"], ['Robert Lewandowski', "56',", "61'"]]</t>
+          <t>[[Raphinha,6,72],[Marc Bernal,18],[Lamine Yamal,45+7 (P)],[Fermín López Marín,51],[Robert Lewandowski,56,61]]</t>
         </is>
       </c>
       <c r="I46" t="n">
@@ -4964,7 +4964,7 @@
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>[['Anthony Elanga', "15',", "28'"]]</t>
+          <t>[[Anthony Elanga,15,28]]</t>
         </is>
       </c>
       <c r="T46" t="n">

</xml_diff>